<commit_message>
new prompt and more cleaned config list
</commit_message>
<xml_diff>
--- a/systeme_de_Classification_Intelligent_des_emails/emails_output/emails.xlsx
+++ b/systeme_de_Classification_Intelligent_des_emails/emails_output/emails.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>UID</t>
   </si>
@@ -25,30 +25,52 @@
     <t>Attachments</t>
   </si>
   <si>
-    <t xml:space="preserve">---------- Forwarded message ---------_x000D_
-From: yessine tony &lt;yessinetony@gmail.com&gt;_x000D_
-Date: Mon, 6 Apr 2026 at 10:22_x000D_
-Subject: nigga_x000D_
-To: Yessineht@gmail.com &lt;Yessineht@gmail.com&gt;_x000D_
+    <t>19</t>
+  </si>
+  <si>
+    <t>---------- Forwarded message ---------_x005F_x000D_
+From: yessine tony &lt;yessinetony@gmail.com&gt;_x005F_x000D_
+Date: Mon, 6 Apr 2026 at 10:22_x005F_x000D_
+Subject: nigga_x005F_x000D_
+To: Yessineht@gmail.com &lt;Yessineht@gmail.com&gt;_x005F_x000D_
+_x005F_x000D_
+_x005F_x000D_
+this is a test for the attatchement</t>
+  </si>
+  <si>
+    <t>Yessine Ht &lt;yessineht@gmail.com&gt;
+Bonjour,_x000D_
 _x000D_
+Je vous écris afin de vous demander l’autorisation de prendre un congé._x000D_
 _x000D_
-this is a test for the attatchement</t>
+Durant cette période, je veillerai à ce que toutes mes tâches en cours_x000D_
+soient organisées ou transmises afin d’assurer la continuité du travail._x000D_
+_x000D_
+Je reste bien entendu disponible pour toute information complémentaire et_x000D_
+je vous remercie par avance pour votre compréhension._x000D_
+_x000D_
+Cordialement,_x000D_
+yessine haj taieb_x000D_
+developpeur</t>
   </si>
   <si>
     <t>Rapport.pdf; Asset 11.png</t>
+  </si>
+  <si>
+    <t>Doctor_Note_with_Signature.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -78,15 +100,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -374,11 +388,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -389,19 +403,28 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>